<commit_message>
Sync flatfiles from remote location
</commit_message>
<xml_diff>
--- a/scripts/flat-files/SailingPackages/SailingPackage.xlsx
+++ b/scripts/flat-files/SailingPackages/SailingPackage.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="29127"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="30126"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://celestyalepe.sharepoint.com/sites/CommercialExcellence-ToolingTech/Shared Documents/General/6. File_Share/Web Cache/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="138" documentId="11_BC4EB32AFE82BCE1C851F3599A4DF0B49E5EEC3C" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{5FDC1F25-D581-42D5-BF9F-B6D2F3388EDA}"/>
+  <xr:revisionPtr revIDLastSave="163" documentId="11_BC4EB32AFE82BCE1C851F3599A4DF0B49E5EEC3C" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{B3F4DB15-5ADB-4C6C-8B35-3678F17F5A9F}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -30,6 +30,8 @@
         <xcalcf:feature name="microsoft.com:FV"/>
         <xcalcf:feature name="microsoft.com:CNMTM"/>
         <xcalcf:feature name="microsoft.com:LET_WF"/>
+        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
+        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
       </xcalcf:calcFeatures>
     </ext>
   </extLst>
@@ -54,22 +56,22 @@
     <t>Required</t>
   </si>
   <si>
+    <t>PIR</t>
+  </si>
+  <si>
+    <t>MEDICONSEW</t>
+  </si>
+  <si>
+    <t>MEDICONSWE</t>
+  </si>
+  <si>
+    <t>MEDICONSEWV</t>
+  </si>
+  <si>
+    <t>MEDICONSWEV</t>
+  </si>
+  <si>
     <t>ABD</t>
-  </si>
-  <si>
-    <t>PIR</t>
-  </si>
-  <si>
-    <t>MEDICONSEW</t>
-  </si>
-  <si>
-    <t>MEDICONSWE</t>
-  </si>
-  <si>
-    <t>MEDICONSEWV</t>
-  </si>
-  <si>
-    <t>MEDICONSWEV</t>
   </si>
   <si>
     <t>LAV</t>
@@ -175,7 +177,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="2" x14ac:knownFonts="1">
+  <fonts count="2">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -550,15 +552,15 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:E39"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="14.45"/>
   <cols>
-    <col min="1" max="1" width="12.33203125" bestFit="1" customWidth="1"/>
-    <col min="2" max="3" width="12.33203125" customWidth="1"/>
-    <col min="4" max="4" width="27.6640625" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="19.109375" customWidth="1"/>
+    <col min="1" max="1" width="12.28515625" bestFit="1" customWidth="1"/>
+    <col min="2" max="3" width="12.28515625" customWidth="1"/>
+    <col min="4" max="4" width="27.7109375" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="19.140625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:5">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -575,77 +577,77 @@
         <v>4</v>
       </c>
     </row>
-    <row r="2" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:5">
       <c r="A2" t="s">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="B2" t="s">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="C2">
         <v>14</v>
       </c>
       <c r="D2" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="E2">
         <v>1</v>
       </c>
     </row>
-    <row r="3" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:5">
       <c r="A3" t="s">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="B3" t="s">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="C3">
         <v>14</v>
       </c>
       <c r="D3" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="E3">
         <v>1</v>
       </c>
     </row>
-    <row r="4" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:5">
       <c r="A4" t="s">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="B4" t="s">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="C4">
         <v>14</v>
       </c>
       <c r="D4" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="E4">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="5" spans="1:5" x14ac:dyDescent="0.3">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="5" spans="1:5">
       <c r="A5" t="s">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="B5" t="s">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="C5">
         <v>14</v>
       </c>
       <c r="D5" t="s">
+        <v>9</v>
+      </c>
+      <c r="E5">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="6" spans="1:5">
+      <c r="A6" t="s">
         <v>10</v>
-      </c>
-      <c r="E5">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="6" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A6" t="s">
-        <v>5</v>
       </c>
       <c r="B6" t="s">
         <v>11</v>
@@ -657,15 +659,15 @@
         <v>12</v>
       </c>
       <c r="E6">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="7" spans="1:5" x14ac:dyDescent="0.3">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="7" spans="1:5">
       <c r="A7" t="s">
         <v>11</v>
       </c>
       <c r="B7" t="s">
-        <v>5</v>
+        <v>10</v>
       </c>
       <c r="C7">
         <v>14</v>
@@ -674,15 +676,15 @@
         <v>13</v>
       </c>
       <c r="E7">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="8" spans="1:5" x14ac:dyDescent="0.3">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="8" spans="1:5">
       <c r="A8" t="s">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="B8" t="s">
-        <v>5</v>
+        <v>10</v>
       </c>
       <c r="C8">
         <v>14</v>
@@ -691,15 +693,15 @@
         <v>14</v>
       </c>
       <c r="E8">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="9" spans="1:5" x14ac:dyDescent="0.3">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="9" spans="1:5">
       <c r="A9" t="s">
         <v>15</v>
       </c>
       <c r="B9" t="s">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="C9">
         <v>14</v>
@@ -708,10 +710,10 @@
         <v>16</v>
       </c>
       <c r="E9">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="10" spans="1:5" x14ac:dyDescent="0.3">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="10" spans="1:5">
       <c r="A10" t="s">
         <v>11</v>
       </c>
@@ -728,7 +730,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="11" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:5">
       <c r="A11" t="s">
         <v>11</v>
       </c>
@@ -745,7 +747,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="12" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:5">
       <c r="A12" t="s">
         <v>11</v>
       </c>
@@ -762,7 +764,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="13" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:5">
       <c r="A13" t="s">
         <v>11</v>
       </c>
@@ -779,12 +781,12 @@
         <v>1</v>
       </c>
     </row>
-    <row r="14" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:5">
       <c r="A14" t="s">
-        <v>5</v>
+        <v>10</v>
       </c>
       <c r="B14" t="s">
-        <v>5</v>
+        <v>10</v>
       </c>
       <c r="C14">
         <v>3</v>
@@ -793,15 +795,15 @@
         <v>21</v>
       </c>
       <c r="E14">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="15" spans="1:5" x14ac:dyDescent="0.3">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="15" spans="1:5">
       <c r="A15" t="s">
-        <v>5</v>
+        <v>10</v>
       </c>
       <c r="B15" t="s">
-        <v>5</v>
+        <v>10</v>
       </c>
       <c r="C15">
         <v>4</v>
@@ -810,15 +812,15 @@
         <v>22</v>
       </c>
       <c r="E15">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="16" spans="1:5" x14ac:dyDescent="0.3">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="16" spans="1:5">
       <c r="A16" t="s">
-        <v>5</v>
+        <v>10</v>
       </c>
       <c r="B16" t="s">
-        <v>5</v>
+        <v>10</v>
       </c>
       <c r="C16">
         <v>7</v>
@@ -827,15 +829,15 @@
         <v>23</v>
       </c>
       <c r="E16">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="17" spans="1:5" x14ac:dyDescent="0.3">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="17" spans="1:5">
       <c r="A17" t="s">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="B17" t="s">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="C17">
         <v>7</v>
@@ -847,12 +849,12 @@
         <v>1</v>
       </c>
     </row>
-    <row r="18" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="18" spans="1:5">
       <c r="A18" t="s">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="B18" t="s">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="C18">
         <v>7</v>
@@ -864,12 +866,12 @@
         <v>1</v>
       </c>
     </row>
-    <row r="19" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="19" spans="1:5">
       <c r="A19" t="s">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="B19" t="s">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="C19">
         <v>7</v>
@@ -881,7 +883,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="20" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="20" spans="1:5">
       <c r="A20" t="s">
         <v>15</v>
       </c>
@@ -895,10 +897,10 @@
         <v>27</v>
       </c>
       <c r="E20">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="21" spans="1:5" x14ac:dyDescent="0.3">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="21" spans="1:5">
       <c r="A21" t="s">
         <v>28</v>
       </c>
@@ -912,10 +914,10 @@
         <v>29</v>
       </c>
       <c r="E21">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="22" spans="1:5" x14ac:dyDescent="0.3">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="22" spans="1:5">
       <c r="A22" t="s">
         <v>30</v>
       </c>
@@ -929,12 +931,12 @@
         <v>29</v>
       </c>
       <c r="E22">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="23" spans="1:5" x14ac:dyDescent="0.3">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="23" spans="1:5">
       <c r="A23" t="s">
-        <v>5</v>
+        <v>10</v>
       </c>
       <c r="B23" t="s">
         <v>28</v>
@@ -946,15 +948,15 @@
         <v>31</v>
       </c>
       <c r="E23">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="24" spans="1:5" x14ac:dyDescent="0.3">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="24" spans="1:5">
       <c r="A24" t="s">
         <v>28</v>
       </c>
       <c r="B24" t="s">
-        <v>5</v>
+        <v>10</v>
       </c>
       <c r="C24">
         <v>4</v>
@@ -963,10 +965,10 @@
         <v>32</v>
       </c>
       <c r="E24">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="25" spans="1:5" x14ac:dyDescent="0.3">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="25" spans="1:5">
       <c r="A25" t="s">
         <v>15</v>
       </c>
@@ -980,10 +982,10 @@
         <v>33</v>
       </c>
       <c r="E25">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="26" spans="1:5" x14ac:dyDescent="0.3">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="26" spans="1:5">
       <c r="A26" t="s">
         <v>28</v>
       </c>
@@ -997,10 +999,10 @@
         <v>33</v>
       </c>
       <c r="E26">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="27" spans="1:5" x14ac:dyDescent="0.3">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="27" spans="1:5">
       <c r="A27" t="s">
         <v>30</v>
       </c>
@@ -1014,10 +1016,10 @@
         <v>33</v>
       </c>
       <c r="E27">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="28" spans="1:5" x14ac:dyDescent="0.3">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="28" spans="1:5">
       <c r="A28" t="s">
         <v>30</v>
       </c>
@@ -1031,10 +1033,10 @@
         <v>34</v>
       </c>
       <c r="E28">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="29" spans="1:5" x14ac:dyDescent="0.3">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="29" spans="1:5">
       <c r="A29" t="s">
         <v>28</v>
       </c>
@@ -1048,15 +1050,15 @@
         <v>34</v>
       </c>
       <c r="E29">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="30" spans="1:5" x14ac:dyDescent="0.3">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="30" spans="1:5">
       <c r="A30" t="s">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="B30" t="s">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="C30">
         <v>14</v>
@@ -1068,12 +1070,12 @@
         <v>1</v>
       </c>
     </row>
-    <row r="31" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="31" spans="1:5">
       <c r="A31" t="s">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="B31" t="s">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="C31">
         <v>14</v>
@@ -1085,12 +1087,12 @@
         <v>1</v>
       </c>
     </row>
-    <row r="32" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="32" spans="1:5">
       <c r="A32" t="s">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="B32" t="s">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="C32">
         <v>14</v>
@@ -1102,12 +1104,12 @@
         <v>1</v>
       </c>
     </row>
-    <row r="33" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="33" spans="1:5">
       <c r="A33" t="s">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="B33" t="s">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="C33">
         <v>14</v>
@@ -1119,7 +1121,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="34" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="34" spans="1:5">
       <c r="A34" t="s">
         <v>28</v>
       </c>
@@ -1133,10 +1135,10 @@
         <v>39</v>
       </c>
       <c r="E34">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="35" spans="1:5" x14ac:dyDescent="0.3">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="35" spans="1:5">
       <c r="A35" t="s">
         <v>30</v>
       </c>
@@ -1150,10 +1152,10 @@
         <v>39</v>
       </c>
       <c r="E35">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="36" spans="1:5" x14ac:dyDescent="0.3">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="36" spans="1:5">
       <c r="A36" t="s">
         <v>15</v>
       </c>
@@ -1167,10 +1169,10 @@
         <v>40</v>
       </c>
       <c r="E36">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="37" spans="1:5" x14ac:dyDescent="0.3">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="37" spans="1:5">
       <c r="A37" t="s">
         <v>30</v>
       </c>
@@ -1184,10 +1186,10 @@
         <v>41</v>
       </c>
       <c r="E37">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="38" spans="1:5" x14ac:dyDescent="0.3">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="38" spans="1:5">
       <c r="A38" t="s">
         <v>15</v>
       </c>
@@ -1201,15 +1203,15 @@
         <v>42</v>
       </c>
       <c r="E38">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="39" spans="1:5" x14ac:dyDescent="0.3">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="39" spans="1:5">
       <c r="A39" t="s">
-        <v>5</v>
+        <v>10</v>
       </c>
       <c r="B39" t="s">
-        <v>5</v>
+        <v>10</v>
       </c>
       <c r="C39">
         <v>7</v>
@@ -1218,7 +1220,7 @@
         <v>43</v>
       </c>
       <c r="E39">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
   </sheetData>
@@ -1237,17 +1239,6 @@
 </file>
 
 <file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <lcf76f155ced4ddcb4097134ff3c332f xmlns="d8ccb410-e8f8-4e64-923b-36eaccbbdce1">
-      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    </lcf76f155ced4ddcb4097134ff3c332f>
-    <TaxCatchAll xmlns="1f0d39c8-c576-416d-9b8e-2dcd71db641c" xsi:nil="true"/>
-  </documentManagement>
-</p:properties>
-</file>
-
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x010100B9C8A73C1706E040BD7C6C99A3EBF51D" ma:contentTypeVersion="14" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="ee0aab5accfab02ea1f430a064e9a759">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="d8ccb410-e8f8-4e64-923b-36eaccbbdce1" xmlns:ns3="1f0d39c8-c576-416d-9b8e-2dcd71db641c" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="48eb31dbb7594155fb6027d886920afd" ns2:_="" ns3:_="">
     <xsd:import namespace="d8ccb410-e8f8-4e64-923b-36eaccbbdce1"/>
@@ -1476,46 +1467,25 @@
 </ct:contentTypeSchema>
 </file>
 
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="d8ccb410-e8f8-4e64-923b-36eaccbbdce1">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </lcf76f155ced4ddcb4097134ff3c332f>
+    <TaxCatchAll xmlns="1f0d39c8-c576-416d-9b8e-2dcd71db641c" xsi:nil="true"/>
+  </documentManagement>
+</p:properties>
+</file>
+
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{5461E57B-1E5F-4E65-A945-C8A202A07209}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{5461E57B-1E5F-4E65-A945-C8A202A07209}"/>
 </file>
 
 <file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{7D61AE56-39B0-4970-B18D-D4B1AB4585EA}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="d8ccb410-e8f8-4e64-923b-36eaccbbdce1"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/dcmitype/"/>
-    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
-    <ds:schemaRef ds:uri="1f0d39c8-c576-416d-9b8e-2dcd71db641c"/>
-    <ds:schemaRef ds:uri="http://www.w3.org/XML/1998/namespace"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{3958504B-749D-428A-A2D1-778D79B5C7D6}"/>
 </file>
 
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{3958504B-749D-428A-A2D1-778D79B5C7D6}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes"/>
-    <ds:schemaRef ds:uri="http://www.w3.org/2001/XMLSchema"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="d8ccb410-e8f8-4e64-923b-36eaccbbdce1"/>
-    <ds:schemaRef ds:uri="1f0d39c8-c576-416d-9b8e-2dcd71db641c"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{7D61AE56-39B0-4970-B18D-D4B1AB4585EA}"/>
 </file>
</xml_diff>